<commit_message>
Remove edit, add function
</commit_message>
<xml_diff>
--- a/backend/real_data/teachers_information_4.xlsx
+++ b/backend/real_data/teachers_information_4.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\school_timeTable_v2.0\backend\real_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\school_timeTable\backend\real_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{310759A5-507C-4B60-99AB-FD07D3056E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCFCD677-E955-4B08-858E-7F357F692395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11895" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="253">
   <si>
     <t>Mã Giáo Viên</t>
   </si>
@@ -31,9 +31,6 @@
     <t>Số Tiết Dạy Tối Đa 1 Tuần</t>
   </si>
   <si>
-    <t>Tiết Không Thể Dạy</t>
-  </si>
-  <si>
     <t>Phân công dạy môn-lớp</t>
   </si>
   <si>
@@ -685,18 +682,6 @@
     <t>12A12</t>
   </si>
   <si>
-    <t>Nghỉ Thứ 2, thứ 3</t>
-  </si>
-  <si>
-    <t>Nghỉ Thứ 5, thứ 7</t>
-  </si>
-  <si>
-    <t>Nghỉ Tiết 1, Thứ 2,4,6</t>
-  </si>
-  <si>
-    <t>Nghỉ tiết 1, Thứ 3,5,7</t>
-  </si>
-  <si>
     <t>Lê Minh Thành</t>
   </si>
   <si>
@@ -716,12 +701,6 @@
   </si>
   <si>
     <t>QP11-11A6, QP11-11A7, QP11-11A8, QP11-11A9, QP11-11A10, QP11-11A11, QP11-11A12</t>
-  </si>
-  <si>
-    <t>Nghỉ thứ 7</t>
-  </si>
-  <si>
-    <t>Nghỉ tiết 1, Tiết 5</t>
   </si>
   <si>
     <t>TH11-11A1, TH11-11A2, TH11-11A4, TH10-10A5, HĐTN10-10A5, TH11-11A11</t>
@@ -754,9 +733,6 @@
     </r>
   </si>
   <si>
-    <t>Nghỉ Thứ 7, Thứ 5</t>
-  </si>
-  <si>
     <t>NV12-12A3, NV12-12A12, NV10-10A9, NV10-10A12, GDĐP12-12A3, GDĐP12-12A12</t>
   </si>
   <si>
@@ -803,6 +779,27 @@
   </si>
   <si>
     <t>LS12-12A1, LS12-12A3, LS12-12A10, LS11-11A1, LS11-11A5, LS11-11A6, LS11-11A7, LS10-10A2, LS10-10A9,SHL12-12A3</t>
+  </si>
+  <si>
+    <t>Saturday-morning-1,Saturday-morning-2,Saturday-morning-3,Saturday-morning-4,Saturday-morning-5</t>
+  </si>
+  <si>
+    <t>Saturday-morning-1,Saturday-morning-2,Saturday-morning-3,Saturday-morning-4,Saturday-morning-5,Thurday-morning-1,Thurday-morning-2,Thurday-morning-3,Thurday-morning-4,Thurday-morning-5</t>
+  </si>
+  <si>
+    <t>Tuesday-morning-1,Tuesday-morning-2,Tuesday-morning-3,Tuesday-morning-4,Tuesday-morning-5,Monday-morning-1,Monday-morning-2,Monday-morning-3,Monday-morning-4,Monday-morning-5</t>
+  </si>
+  <si>
+    <t>Monday-morning-1,Tuesday-morning-1,Wednesday-morning-1,Thurday-morning-1,Friday-morning-1,Statuday-morning-1,Monday-morning-5,Tuesday-morning-5,Wednesday-morning-5,Thurday-morning-5,Friday-morning-5,Statuday-morning-5</t>
+  </si>
+  <si>
+    <t>Thurday-morning-1,Thurday-morning-2,Thurday-morning-3,Thurday-morning-4,Thurday-morning-5,Saturday-morning-1,Saturday-morning-2,Saturday-morning-3,Saturday-morning-4,Saturday-morning-5</t>
+  </si>
+  <si>
+    <t>Monday-morning-1,Wednesday-morning-1,Friday-morning-1</t>
+  </si>
+  <si>
+    <t>Tuesday-morning-1,Thurday-morning-1,Statuday-morning-1</t>
   </si>
 </sst>
 </file>
@@ -1298,7 +1295,7 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyFont="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1325,6 +1322,15 @@
     </xf>
     <xf numFmtId="164" fontId="28" fillId="0" borderId="10" xfId="40" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="45">
@@ -1681,7 +1687,7 @@
     <col min="2" max="2" width="29.88671875" customWidth="1"/>
     <col min="3" max="3" width="23.88671875" customWidth="1"/>
     <col min="4" max="4" width="13.109375" customWidth="1"/>
-    <col min="5" max="5" width="55.5546875" customWidth="1"/>
+    <col min="5" max="5" width="38.77734375" customWidth="1"/>
     <col min="6" max="6" width="58.5546875" style="7" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -1697,24 +1703,22 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="E1" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="E1" s="1"/>
+      <c r="F1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:7" ht="72">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>7</v>
       </c>
       <c r="C2">
         <v>12</v>
@@ -1722,155 +1726,155 @@
       <c r="D2">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
-        <v>237</v>
+      <c r="E2" s="14" t="s">
+        <v>247</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
       </c>
       <c r="C3">
         <v>16</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="30.6">
       <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>11</v>
       </c>
       <c r="C4">
         <v>14</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="G4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="14.4">
       <c r="A5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="C5">
         <v>14</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G5" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="86.4">
       <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
-      <c r="E6" t="s">
-        <v>233</v>
+      <c r="E6" s="13" t="s">
+        <v>249</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>19</v>
       </c>
       <c r="C7">
         <v>14</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="G7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="14.4">
       <c r="A8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="C8">
         <v>14</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G8" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="14.4">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="72">
       <c r="A9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="C9">
         <v>14</v>
       </c>
-      <c r="E9" t="s">
-        <v>221</v>
+      <c r="E9" s="14" t="s">
+        <v>248</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="C10">
         <v>12</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G10" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="C11">
         <v>16</v>
@@ -1879,66 +1883,66 @@
         <v>1</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="30.6">
       <c r="A12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="C12">
         <v>14</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="G12" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="43.2">
       <c r="A13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="C13">
         <v>16</v>
       </c>
-      <c r="E13" t="s">
-        <v>232</v>
+      <c r="E13" s="13" t="s">
+        <v>246</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="86.4">
       <c r="A14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="C14">
         <v>4</v>
       </c>
-      <c r="E14" t="s">
-        <v>233</v>
+      <c r="E14" s="13" t="s">
+        <v>249</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="3" customFormat="1" ht="30.6">
       <c r="A15" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>13</v>
       </c>
       <c r="C15" s="3">
         <v>16</v>
@@ -1947,15 +1951,15 @@
         <v>1</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="30.6">
       <c r="A16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="C16">
         <v>10</v>
@@ -1964,35 +1968,35 @@
         <v>1</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G16" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="30.6">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="72">
       <c r="A17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="C17">
         <v>14</v>
       </c>
-      <c r="E17" t="s">
-        <v>222</v>
+      <c r="E17" s="13" t="s">
+        <v>250</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
     </row>
     <row r="18" spans="1:7" s="3" customFormat="1" ht="30.6">
       <c r="A18" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>39</v>
       </c>
       <c r="C18" s="3">
         <v>16</v>
@@ -2001,15 +2005,15 @@
         <v>1</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="30.6">
       <c r="A19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" t="s">
         <v>54</v>
-      </c>
-      <c r="B19" t="s">
-        <v>55</v>
       </c>
       <c r="C19">
         <v>10</v>
@@ -2018,148 +2022,148 @@
         <v>4</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="30.6">
       <c r="A20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" t="s">
         <v>56</v>
-      </c>
-      <c r="B20" t="s">
-        <v>57</v>
       </c>
       <c r="C20">
         <v>15</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G20" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="30.6">
       <c r="A21" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" t="s">
         <v>62</v>
-      </c>
-      <c r="B21" t="s">
-        <v>63</v>
       </c>
       <c r="C21">
         <v>13</v>
       </c>
-      <c r="E21" t="s">
-        <v>223</v>
+      <c r="E21" s="13" t="s">
+        <v>251</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="G21" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="30.6">
       <c r="A22" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" t="s">
         <v>64</v>
-      </c>
-      <c r="B22" t="s">
-        <v>65</v>
       </c>
       <c r="C22">
         <v>17</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30.6">
       <c r="A23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B23" t="s">
         <v>68</v>
-      </c>
-      <c r="B23" t="s">
-        <v>69</v>
       </c>
       <c r="C23">
         <v>15</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G23" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="24" spans="1:7" s="3" customFormat="1">
       <c r="A24" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>40</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>41</v>
       </c>
       <c r="C24" s="3">
         <v>14</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="30.6">
       <c r="A25" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" t="s">
         <v>52</v>
-      </c>
-      <c r="B25" t="s">
-        <v>53</v>
       </c>
       <c r="C25">
         <v>11</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="G25" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="30.6">
       <c r="A26" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" t="s">
         <v>48</v>
-      </c>
-      <c r="B26" t="s">
-        <v>49</v>
       </c>
       <c r="C26">
         <v>13</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G26" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="30.6">
       <c r="A27" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" t="s">
         <v>50</v>
-      </c>
-      <c r="B27" t="s">
-        <v>51</v>
       </c>
       <c r="C27">
         <v>14</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="G27" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="30.6">
       <c r="A28" t="s">
+        <v>69</v>
+      </c>
+      <c r="B28" t="s">
         <v>70</v>
-      </c>
-      <c r="B28" t="s">
-        <v>71</v>
       </c>
       <c r="C28">
         <v>12</v>
@@ -2168,329 +2172,329 @@
         <v>1</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G28" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="30.6">
       <c r="A29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B29" t="s">
         <v>74</v>
-      </c>
-      <c r="B29" t="s">
-        <v>75</v>
       </c>
       <c r="C29">
         <v>17</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="30" spans="1:7" s="3" customFormat="1" ht="30.6">
       <c r="A30" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>42</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>43</v>
       </c>
       <c r="C30" s="3">
         <v>14</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" t="s">
         <v>46</v>
-      </c>
-      <c r="B31" t="s">
-        <v>47</v>
       </c>
       <c r="C31">
         <v>7</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="30.6">
       <c r="A32" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" t="s">
         <v>58</v>
-      </c>
-      <c r="B32" t="s">
-        <v>59</v>
       </c>
       <c r="C32">
         <v>12</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="G32" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" t="s">
+        <v>65</v>
+      </c>
+      <c r="B33" t="s">
         <v>66</v>
-      </c>
-      <c r="B33" t="s">
-        <v>67</v>
       </c>
       <c r="C33">
         <v>2</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="34" spans="1:7" s="3" customFormat="1" ht="45.6">
       <c r="A34" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B34" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>45</v>
       </c>
       <c r="C34" s="3">
         <v>20</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="45.6">
       <c r="A35" t="s">
+        <v>59</v>
+      </c>
+      <c r="B35" t="s">
         <v>60</v>
-      </c>
-      <c r="B35" t="s">
-        <v>61</v>
       </c>
       <c r="C35">
         <v>14</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="G35" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="30.6">
       <c r="A36" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" t="s">
         <v>72</v>
-      </c>
-      <c r="B36" t="s">
-        <v>73</v>
       </c>
       <c r="C36">
         <v>14</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G36" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="37" spans="1:7" s="3" customFormat="1" ht="30.6">
       <c r="A37" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>77</v>
       </c>
       <c r="C37" s="3">
         <v>17</v>
       </c>
-      <c r="E37" s="3" t="s">
-        <v>224</v>
+      <c r="E37" s="15" t="s">
+        <v>252</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="45.6">
       <c r="A38" t="s">
+        <v>77</v>
+      </c>
+      <c r="B38" t="s">
         <v>78</v>
-      </c>
-      <c r="B38" t="s">
-        <v>79</v>
       </c>
       <c r="C38">
         <v>18</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G38" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="45.6">
       <c r="A39" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" t="s">
         <v>80</v>
-      </c>
-      <c r="B39" t="s">
-        <v>81</v>
       </c>
       <c r="C39">
         <v>18</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="G39" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="30.6">
       <c r="A40" t="s">
+        <v>81</v>
+      </c>
+      <c r="B40" t="s">
         <v>82</v>
-      </c>
-      <c r="B40" t="s">
-        <v>83</v>
       </c>
       <c r="C40">
         <v>14</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G40" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="30.6">
       <c r="A41" t="s">
+        <v>83</v>
+      </c>
+      <c r="B41" t="s">
         <v>84</v>
-      </c>
-      <c r="B41" t="s">
-        <v>85</v>
       </c>
       <c r="C41">
         <v>17</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="G41" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="45.6">
       <c r="A42" t="s">
+        <v>85</v>
+      </c>
+      <c r="B42" t="s">
         <v>86</v>
-      </c>
-      <c r="B42" t="s">
-        <v>87</v>
       </c>
       <c r="C42">
         <v>16</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="G42" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="30.6">
       <c r="A43" t="s">
+        <v>87</v>
+      </c>
+      <c r="B43" t="s">
         <v>88</v>
-      </c>
-      <c r="B43" t="s">
-        <v>89</v>
       </c>
       <c r="C43">
         <v>17</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G43" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="45.6">
       <c r="A44" t="s">
+        <v>89</v>
+      </c>
+      <c r="B44" t="s">
         <v>90</v>
-      </c>
-      <c r="B44" t="s">
-        <v>91</v>
       </c>
       <c r="C44">
         <v>18</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="45.6">
       <c r="A45" t="s">
+        <v>91</v>
+      </c>
+      <c r="B45" t="s">
         <v>92</v>
-      </c>
-      <c r="B45" t="s">
-        <v>93</v>
       </c>
       <c r="C45">
         <v>18</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="G45" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="45.6">
       <c r="A46" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B46" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C46">
         <v>12</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="47" spans="1:7" s="3" customFormat="1" ht="30.6">
       <c r="A47" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B47" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>97</v>
       </c>
       <c r="C47" s="3">
         <v>14</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="30.6">
       <c r="A48" t="s">
+        <v>97</v>
+      </c>
+      <c r="B48" t="s">
         <v>98</v>
-      </c>
-      <c r="B48" t="s">
-        <v>99</v>
       </c>
       <c r="C48">
         <v>16</v>
@@ -2499,117 +2503,117 @@
         <v>1</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="30.6">
       <c r="A49" t="s">
+        <v>101</v>
+      </c>
+      <c r="B49" t="s">
         <v>102</v>
-      </c>
-      <c r="B49" t="s">
-        <v>103</v>
       </c>
       <c r="C49">
         <v>17</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="43.2">
       <c r="A50" t="s">
+        <v>103</v>
+      </c>
+      <c r="B50" t="s">
         <v>104</v>
-      </c>
-      <c r="B50" t="s">
-        <v>105</v>
       </c>
       <c r="C50">
         <v>11</v>
       </c>
-      <c r="E50" t="s">
-        <v>232</v>
+      <c r="E50" s="13" t="s">
+        <v>246</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G50" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="30.6">
       <c r="A51" t="s">
+        <v>105</v>
+      </c>
+      <c r="B51" t="s">
         <v>106</v>
-      </c>
-      <c r="B51" t="s">
-        <v>107</v>
       </c>
       <c r="C51">
         <v>14</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G51" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="30.6">
       <c r="A52" t="s">
+        <v>107</v>
+      </c>
+      <c r="B52" t="s">
         <v>108</v>
-      </c>
-      <c r="B52" t="s">
-        <v>109</v>
       </c>
       <c r="C52">
         <v>14</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G52" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="30.6">
       <c r="A53" t="s">
+        <v>109</v>
+      </c>
+      <c r="B53" t="s">
         <v>110</v>
-      </c>
-      <c r="B53" t="s">
-        <v>111</v>
       </c>
       <c r="C53">
         <v>14</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G53" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="30.6">
       <c r="A54" t="s">
+        <v>111</v>
+      </c>
+      <c r="B54" t="s">
         <v>112</v>
-      </c>
-      <c r="B54" t="s">
-        <v>113</v>
       </c>
       <c r="C54">
         <v>14</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="G54" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="30.6">
       <c r="A55" t="s">
+        <v>113</v>
+      </c>
+      <c r="B55" t="s">
         <v>114</v>
-      </c>
-      <c r="B55" t="s">
-        <v>115</v>
       </c>
       <c r="C55">
         <v>16</v>
@@ -2618,91 +2622,91 @@
         <v>1</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
     </row>
     <row r="56" spans="1:7" s="3" customFormat="1" ht="45.6">
       <c r="A56" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B56" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>117</v>
       </c>
       <c r="C56" s="3">
         <v>22</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="57" spans="1:7">
       <c r="A57" t="s">
+        <v>119</v>
+      </c>
+      <c r="B57" t="s">
         <v>120</v>
-      </c>
-      <c r="B57" t="s">
-        <v>121</v>
       </c>
       <c r="C57">
         <v>2</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="45.6">
       <c r="A58" t="s">
+        <v>129</v>
+      </c>
+      <c r="B58" t="s">
         <v>130</v>
-      </c>
-      <c r="B58" t="s">
-        <v>131</v>
       </c>
       <c r="C58">
         <v>15</v>
       </c>
       <c r="F58" s="8" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="G58" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="30.6">
       <c r="A59" t="s">
+        <v>131</v>
+      </c>
+      <c r="B59" t="s">
         <v>132</v>
-      </c>
-      <c r="B59" t="s">
-        <v>133</v>
       </c>
       <c r="C59">
         <v>14</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G59" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="30.6">
       <c r="A60" t="s">
+        <v>135</v>
+      </c>
+      <c r="B60" t="s">
         <v>136</v>
-      </c>
-      <c r="B60" t="s">
-        <v>137</v>
       </c>
       <c r="C60">
         <v>11</v>
       </c>
       <c r="F60" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="61" spans="1:7" s="3" customFormat="1" ht="30.6">
       <c r="A61" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B61" s="3" t="s">
         <v>124</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>125</v>
       </c>
       <c r="C61" s="3">
         <v>16</v>
@@ -2711,15 +2715,15 @@
         <v>1</v>
       </c>
       <c r="F61" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="30.6">
       <c r="A62" t="s">
+        <v>125</v>
+      </c>
+      <c r="B62" t="s">
         <v>126</v>
-      </c>
-      <c r="B62" t="s">
-        <v>127</v>
       </c>
       <c r="C62">
         <v>13</v>
@@ -2728,15 +2732,15 @@
         <v>4</v>
       </c>
       <c r="F62" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="30.6">
       <c r="A63" t="s">
+        <v>127</v>
+      </c>
+      <c r="B63" t="s">
         <v>128</v>
-      </c>
-      <c r="B63" t="s">
-        <v>129</v>
       </c>
       <c r="C63">
         <v>14</v>
@@ -2745,15 +2749,15 @@
         <v>2</v>
       </c>
       <c r="F63" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="64" spans="1:7">
       <c r="A64" t="s">
+        <v>133</v>
+      </c>
+      <c r="B64" t="s">
         <v>134</v>
-      </c>
-      <c r="B64" t="s">
-        <v>135</v>
       </c>
       <c r="C64">
         <v>12</v>
@@ -2762,15 +2766,15 @@
         <v>5</v>
       </c>
       <c r="F64" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="65" spans="1:6" s="3" customFormat="1" ht="45.6">
       <c r="A65" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B65" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>119</v>
       </c>
       <c r="C65" s="3">
         <v>16</v>
@@ -2779,60 +2783,60 @@
         <v>1</v>
       </c>
       <c r="F65" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="30.6">
       <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66" t="s">
         <v>94</v>
       </c>
-      <c r="B66" t="s">
-        <v>95</v>
-      </c>
       <c r="F66" s="8" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="30.6">
       <c r="A67" t="s">
+        <v>99</v>
+      </c>
+      <c r="B67" t="s">
         <v>100</v>
       </c>
-      <c r="B67" t="s">
-        <v>101</v>
-      </c>
       <c r="F67" s="8" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="60.6">
       <c r="A68" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" t="s">
         <v>122</v>
-      </c>
-      <c r="B68" t="s">
-        <v>123</v>
       </c>
       <c r="C68">
         <v>17</v>
       </c>
-      <c r="E68" t="s">
-        <v>232</v>
+      <c r="E68" s="13" t="s">
+        <v>246</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="30.6">
       <c r="A69" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="B69" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="C69">
         <v>7</v>
       </c>
       <c r="F69" s="9" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>